<commit_message>
Update old_new_pl.xlsx data file
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/data/old_new_pl.xlsx
+++ b/frontend/public/data/old_new_pl.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\업무인수인계\6.실적보고\2025년\stodashboard\frontend\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57752B8E-1142-4A00-973E-11D1091FF1A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F66E3F87-EF96-47F1-A9D5-38DD5D392909}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="15" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{0C279A8B-39A3-4ED4-B4B9-CA68FBFF28CA}"/>
   </bookViews>
@@ -19897,7 +19897,10 @@
         <f t="shared" si="15"/>
         <v>-1937642.2172558359</v>
       </c>
-      <c r="H65" s="17"/>
+      <c r="H65" s="17">
+        <f>G65-old!G65</f>
+        <v>-3796987.2655365765</v>
+      </c>
       <c r="I65" s="17"/>
     </row>
     <row r="66" spans="2:11" ht="15" customHeight="1">

</xml_diff>